<commit_message>
Add Excel launch button templates
</commit_message>
<xml_diff>
--- a/data/use_cases/uc01_122_same_contract_result.xlsx
+++ b/data/use_cases/uc01_122_same_contract_result.xlsx
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="5">
@@ -851,7 +851,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.247н / группа 3 / уровень 1 / оклад 40400</t>
+          <t>3.247н / группа 3 / уровень 1</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.247н / группа 3 / уровень 1 / оклад 40400</t>
+          <t>3.247н / группа 3 / уровень 1</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1979,7 +1979,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Дата построения 03.07.2026</t>
+          <t>Дата построения 10.07.2026</t>
         </is>
       </c>
     </row>

</xml_diff>